<commit_message>
backtest and updated stock report data.
</commit_message>
<xml_diff>
--- a/final_result/stock/quality_momentum_rs_lv.xlsx
+++ b/final_result/stock/quality_momentum_rs_lv.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -496,32 +496,32 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Largecap</t>
+          <t>Midcap</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>7230</v>
+        <v>5392</v>
       </c>
       <c r="F2" t="n">
-        <v>7230</v>
+        <v>5392</v>
       </c>
       <c r="G2" t="n">
-        <v>324.97</v>
+        <v>232.54</v>
       </c>
       <c r="H2" t="n">
-        <v>1.9</v>
+        <v>1.36</v>
       </c>
       <c r="I2" t="n">
-        <v>19.74</v>
+        <v>4.88</v>
       </c>
       <c r="J2" t="n">
-        <v>43.94</v>
+        <v>23.58</v>
       </c>
       <c r="K2" t="n">
-        <v>40.27</v>
+        <v>23.23</v>
       </c>
       <c r="L2" t="n">
-        <v>28.89</v>
+        <v>42.28</v>
       </c>
     </row>
     <row r="3">
@@ -530,7 +530,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -544,28 +544,28 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5266.4</v>
+        <v>9152.5</v>
       </c>
       <c r="F3" t="n">
-        <v>5266.4</v>
+        <v>9152.5</v>
       </c>
       <c r="G3" t="n">
-        <v>319.36</v>
+        <v>429.37</v>
       </c>
       <c r="H3" t="n">
-        <v>1.71</v>
+        <v>2.19</v>
       </c>
       <c r="I3" t="n">
-        <v>14.26</v>
+        <v>11.85</v>
       </c>
       <c r="J3" t="n">
-        <v>31.47</v>
+        <v>17.13</v>
       </c>
       <c r="K3" t="n">
-        <v>23.44</v>
+        <v>19.17</v>
       </c>
       <c r="L3" t="n">
-        <v>49.65</v>
+        <v>35.77</v>
       </c>
     </row>
     <row r="4">
@@ -574,12 +574,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FINCABLES</t>
+          <t>ABSLAMC</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Capital Goods</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -588,28 +588,28 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>990.55</v>
+        <v>1030.4</v>
       </c>
       <c r="F4" t="n">
-        <v>990.55</v>
+        <v>1030.4</v>
       </c>
       <c r="G4" t="n">
-        <v>40.49</v>
+        <v>60.71</v>
       </c>
       <c r="H4" t="n">
-        <v>1.77</v>
+        <v>2.1</v>
       </c>
       <c r="I4" t="n">
-        <v>24.01</v>
+        <v>-3.54</v>
       </c>
       <c r="J4" t="n">
-        <v>36.46</v>
+        <v>19.7</v>
       </c>
       <c r="K4" t="n">
-        <v>26.1</v>
+        <v>39.8</v>
       </c>
       <c r="L4" t="n">
-        <v>11.29</v>
+        <v>21.39</v>
       </c>
     </row>
     <row r="5">
@@ -618,42 +618,42 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ABSLAMC</t>
+          <t>KEI</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Capital Goods</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Smallcap</t>
+          <t>Midcap</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1015.2</v>
+        <v>5117.5</v>
       </c>
       <c r="F5" t="n">
-        <v>1015.2</v>
+        <v>5117.5</v>
       </c>
       <c r="G5" t="n">
-        <v>52.93</v>
+        <v>249.05</v>
       </c>
       <c r="H5" t="n">
-        <v>2.25</v>
+        <v>2.02</v>
       </c>
       <c r="I5" t="n">
-        <v>12.62</v>
+        <v>5.75</v>
       </c>
       <c r="J5" t="n">
-        <v>30.14</v>
+        <v>11.11</v>
       </c>
       <c r="K5" t="n">
-        <v>25.35</v>
+        <v>25.79</v>
       </c>
       <c r="L5" t="n">
-        <v>19.14</v>
+        <v>33.39</v>
       </c>
     </row>
     <row r="6">
@@ -662,42 +662,42 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Automobile and Auto Components</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Midcap</t>
+          <t>Smallcap</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>607.25</v>
+        <v>2140.4</v>
       </c>
       <c r="F6" t="n">
-        <v>607.25</v>
+        <v>2140.4</v>
       </c>
       <c r="G6" t="n">
-        <v>140.5</v>
+        <v>63.42</v>
       </c>
       <c r="H6" t="n">
-        <v>2.31</v>
+        <v>1.48</v>
       </c>
       <c r="I6" t="n">
-        <v>22.12</v>
+        <v>7.13</v>
       </c>
       <c r="J6" t="n">
-        <v>23.3</v>
+        <v>12.96</v>
       </c>
       <c r="K6" t="n">
-        <v>25.78</v>
+        <v>18.42</v>
       </c>
       <c r="L6" t="n">
-        <v>29.77</v>
+        <v>27.42</v>
       </c>
     </row>
     <row r="7">
@@ -706,42 +706,42 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KEI</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Capital Goods</t>
+          <t>Oil Gas &amp; Consumable Fuels</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Midcap</t>
+          <t>Largecap</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>4857.5</v>
+        <v>462.2</v>
       </c>
       <c r="F7" t="n">
-        <v>4857.5</v>
+        <v>462.2</v>
       </c>
       <c r="G7" t="n">
-        <v>174.65</v>
+        <v>514.5</v>
       </c>
       <c r="H7" t="n">
-        <v>2.15</v>
+        <v>1.42</v>
       </c>
       <c r="I7" t="n">
-        <v>17.48</v>
+        <v>5.34</v>
       </c>
       <c r="J7" t="n">
-        <v>25.22</v>
+        <v>10.65</v>
       </c>
       <c r="K7" t="n">
-        <v>19.67</v>
+        <v>21.17</v>
       </c>
       <c r="L7" t="n">
-        <v>25.28</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="8">
@@ -764,28 +764,28 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>90.37</v>
+        <v>91.41</v>
       </c>
       <c r="F8" t="n">
-        <v>90.37</v>
+        <v>91.41</v>
       </c>
       <c r="G8" t="n">
-        <v>238.59</v>
+        <v>208.12</v>
       </c>
       <c r="H8" t="n">
-        <v>1.45</v>
+        <v>1.84</v>
       </c>
       <c r="I8" t="n">
-        <v>15.61</v>
+        <v>1.82</v>
       </c>
       <c r="J8" t="n">
-        <v>14.23</v>
+        <v>10.21</v>
       </c>
       <c r="K8" t="n">
-        <v>24.77</v>
+        <v>22.04</v>
       </c>
       <c r="L8" t="n">
-        <v>31.78</v>
+        <v>34.38</v>
       </c>
     </row>
     <row r="9">
@@ -794,42 +794,42 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>OFSS</t>
+          <t>GPIL</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Capital Goods</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Midcap</t>
+          <t>Smallcap</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>9455.610000000001</v>
+        <v>287.9</v>
       </c>
       <c r="F9" t="n">
-        <v>9726.5</v>
+        <v>287.9</v>
       </c>
       <c r="G9" t="n">
-        <v>334.75</v>
+        <v>68.44</v>
       </c>
       <c r="H9" t="n">
-        <v>2.26</v>
+        <v>1.93</v>
       </c>
       <c r="I9" t="n">
-        <v>41.31</v>
+        <v>-5.78</v>
       </c>
       <c r="J9" t="n">
-        <v>21.39</v>
+        <v>11.5</v>
       </c>
       <c r="K9" t="n">
-        <v>14.83</v>
+        <v>7.27</v>
       </c>
       <c r="L9" t="n">
-        <v>14.73</v>
+        <v>53.99</v>
       </c>
     </row>
     <row r="10">
@@ -838,42 +838,42 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GPIL</t>
+          <t>AJANTPHARM</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Capital Goods</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Smallcap</t>
+          <t>Midcap</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>296.3</v>
+        <v>3177.2</v>
       </c>
       <c r="F10" t="n">
-        <v>296.3</v>
+        <v>3177.2</v>
       </c>
       <c r="G10" t="n">
-        <v>97.48999999999999</v>
+        <v>41.84</v>
       </c>
       <c r="H10" t="n">
-        <v>2.02</v>
+        <v>2.12</v>
       </c>
       <c r="I10" t="n">
-        <v>6.33</v>
+        <v>13.87</v>
       </c>
       <c r="J10" t="n">
-        <v>15.2</v>
+        <v>9.26</v>
       </c>
       <c r="K10" t="n">
-        <v>10.16</v>
+        <v>23.26</v>
       </c>
       <c r="L10" t="n">
-        <v>57.53</v>
+        <v>22.67</v>
       </c>
     </row>
     <row r="11">
@@ -882,42 +882,42 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>TIMKEN</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Oil Gas &amp; Consumable Fuels</t>
+          <t>Capital Goods</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Largecap</t>
+          <t>Smallcap</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>481.45</v>
+        <v>3531.2</v>
       </c>
       <c r="F11" t="n">
-        <v>481.45</v>
+        <v>3531.2</v>
       </c>
       <c r="G11" t="n">
-        <v>578.89</v>
+        <v>20.59</v>
       </c>
       <c r="H11" t="n">
-        <v>1.7</v>
+        <v>1.63</v>
       </c>
       <c r="I11" t="n">
-        <v>7.13</v>
+        <v>0.7</v>
       </c>
       <c r="J11" t="n">
-        <v>9.859999999999999</v>
+        <v>10.57</v>
       </c>
       <c r="K11" t="n">
-        <v>28.01</v>
+        <v>15.8</v>
       </c>
       <c r="L11" t="n">
-        <v>35.32</v>
+        <v>21.85</v>
       </c>
     </row>
     <row r="12">
@@ -940,28 +940,28 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1458.6</v>
+        <v>1430.5</v>
       </c>
       <c r="F12" t="n">
-        <v>1458.6</v>
+        <v>1430.5</v>
       </c>
       <c r="G12" t="n">
-        <v>338.54</v>
+        <v>391.59</v>
       </c>
       <c r="H12" t="n">
-        <v>1.79</v>
+        <v>1.83</v>
       </c>
       <c r="I12" t="n">
-        <v>23.53</v>
+        <v>11.27</v>
       </c>
       <c r="J12" t="n">
-        <v>13.47</v>
+        <v>9.59</v>
       </c>
       <c r="K12" t="n">
-        <v>15.38</v>
+        <v>12.52</v>
       </c>
       <c r="L12" t="n">
-        <v>28.94</v>
+        <v>31.16</v>
       </c>
     </row>
     <row r="13">
@@ -970,7 +970,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>ZYDUSLIFE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -980,32 +980,32 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Smallcap</t>
+          <t>Largecap</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2043.4</v>
+        <v>1011.7</v>
       </c>
       <c r="F13" t="n">
-        <v>2043.4</v>
+        <v>1011.7</v>
       </c>
       <c r="G13" t="n">
-        <v>60.6</v>
+        <v>95.95999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>1.25</v>
+        <v>1.99</v>
       </c>
       <c r="I13" t="n">
-        <v>1.72</v>
+        <v>7.18</v>
       </c>
       <c r="J13" t="n">
-        <v>10.81</v>
+        <v>12.62</v>
       </c>
       <c r="K13" t="n">
-        <v>22</v>
+        <v>6.34</v>
       </c>
       <c r="L13" t="n">
-        <v>20.9</v>
+        <v>8.07</v>
       </c>
     </row>
     <row r="14">
@@ -1014,42 +1014,42 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Capital Goods</t>
+          <t>Fast Moving Consumer Goods</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Smallcap</t>
+          <t>Midcap</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>553.5</v>
+        <v>841.15</v>
       </c>
       <c r="F14" t="n">
-        <v>553.5</v>
+        <v>841.15</v>
       </c>
       <c r="G14" t="n">
-        <v>26.79</v>
+        <v>147.38</v>
       </c>
       <c r="H14" t="n">
-        <v>1.59</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>15.53</v>
+        <v>11.07</v>
       </c>
       <c r="J14" t="n">
-        <v>28.33</v>
+        <v>9.18</v>
       </c>
       <c r="K14" t="n">
-        <v>11.39</v>
+        <v>16.67</v>
       </c>
       <c r="L14" t="n">
-        <v>-3.42</v>
+        <v>19.49</v>
       </c>
     </row>
     <row r="15">
@@ -1058,12 +1058,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Capital Goods</t>
+          <t>Automobile and Auto Components</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1072,28 +1072,28 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>8110.5</v>
+        <v>573.55</v>
       </c>
       <c r="F15" t="n">
-        <v>8110.5</v>
+        <v>573.55</v>
       </c>
       <c r="G15" t="n">
-        <v>327.87</v>
+        <v>168.91</v>
       </c>
       <c r="H15" t="n">
-        <v>1.98</v>
+        <v>2.14</v>
       </c>
       <c r="I15" t="n">
-        <v>17.12</v>
+        <v>-3.42</v>
       </c>
       <c r="J15" t="n">
-        <v>17.07</v>
+        <v>6.61</v>
       </c>
       <c r="K15" t="n">
-        <v>8</v>
+        <v>15.6</v>
       </c>
       <c r="L15" t="n">
-        <v>20.43</v>
+        <v>29.31</v>
       </c>
     </row>
     <row r="16">
@@ -1102,42 +1102,42 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TIMKEN</t>
+          <t>VBL</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Capital Goods</t>
+          <t>Fast Moving Consumer Goods</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Smallcap</t>
+          <t>Largecap</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>3428.8</v>
+        <v>503.8</v>
       </c>
       <c r="F16" t="n">
-        <v>3428.8</v>
+        <v>503.8</v>
       </c>
       <c r="G16" t="n">
-        <v>18.22</v>
+        <v>392.58</v>
       </c>
       <c r="H16" t="n">
-        <v>2.01</v>
+        <v>2.16</v>
       </c>
       <c r="I16" t="n">
-        <v>2.67</v>
+        <v>6.41</v>
       </c>
       <c r="J16" t="n">
-        <v>14.87</v>
+        <v>10.51</v>
       </c>
       <c r="K16" t="n">
-        <v>13.46</v>
+        <v>9.93</v>
       </c>
       <c r="L16" t="n">
-        <v>-1.42</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="17">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TIINDIA</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1156,32 +1156,32 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Midcap</t>
+          <t>Largecap</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>2947.9</v>
+        <v>10377.5</v>
       </c>
       <c r="F17" t="n">
-        <v>2947.9</v>
+        <v>10377.5</v>
       </c>
       <c r="G17" t="n">
-        <v>94.42</v>
+        <v>424.44</v>
       </c>
       <c r="H17" t="n">
-        <v>2.01</v>
+        <v>1.71</v>
       </c>
       <c r="I17" t="n">
-        <v>14.58</v>
+        <v>6.18</v>
       </c>
       <c r="J17" t="n">
-        <v>29.36</v>
+        <v>5.15</v>
       </c>
       <c r="K17" t="n">
-        <v>-5.6</v>
+        <v>17.02</v>
       </c>
       <c r="L17" t="n">
-        <v>2.13</v>
+        <v>26.19</v>
       </c>
     </row>
     <row r="18">
@@ -1190,12 +1190,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HINDZINC</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Metals &amp; Mining</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1204,28 +1204,28 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>595.95</v>
+        <v>6760.5</v>
       </c>
       <c r="F18" t="n">
-        <v>595.95</v>
+        <v>6760.5</v>
       </c>
       <c r="G18" t="n">
-        <v>363.95</v>
+        <v>191.04</v>
       </c>
       <c r="H18" t="n">
-        <v>2.31</v>
+        <v>1.21</v>
       </c>
       <c r="I18" t="n">
-        <v>15.71</v>
+        <v>7.42</v>
       </c>
       <c r="J18" t="n">
-        <v>-14.31</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>28.79</v>
+        <v>3.38</v>
       </c>
       <c r="L18" t="n">
-        <v>38.17</v>
+        <v>10.26</v>
       </c>
     </row>
     <row r="19">
@@ -1234,42 +1234,42 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>VBL</t>
+          <t>TIINDIA</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fast Moving Consumer Goods</t>
+          <t>Automobile and Auto Components</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Largecap</t>
+          <t>Midcap</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>513.7</v>
+        <v>2850.3</v>
       </c>
       <c r="F19" t="n">
-        <v>513.7</v>
+        <v>2850.3</v>
       </c>
       <c r="G19" t="n">
-        <v>430.42</v>
+        <v>121.17</v>
       </c>
       <c r="H19" t="n">
-        <v>2.34</v>
+        <v>2.26</v>
       </c>
       <c r="I19" t="n">
-        <v>28.13</v>
+        <v>2.15</v>
       </c>
       <c r="J19" t="n">
-        <v>9.91</v>
+        <v>16.33</v>
       </c>
       <c r="K19" t="n">
-        <v>13.36</v>
+        <v>-6.02</v>
       </c>
       <c r="L19" t="n">
-        <v>8</v>
+        <v>-1.14</v>
       </c>
     </row>
     <row r="20">
@@ -1278,42 +1278,42 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Automobile and Auto Components</t>
+          <t>Capital Goods</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Largecap</t>
+          <t>Smallcap</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>9994</v>
+        <v>523.25</v>
       </c>
       <c r="F20" t="n">
-        <v>9994</v>
+        <v>523.25</v>
       </c>
       <c r="G20" t="n">
-        <v>376.39</v>
+        <v>17.57</v>
       </c>
       <c r="H20" t="n">
-        <v>1.69</v>
+        <v>1.75</v>
       </c>
       <c r="I20" t="n">
-        <v>12.35</v>
+        <v>-4.72</v>
       </c>
       <c r="J20" t="n">
-        <v>5.94</v>
+        <v>5.18</v>
       </c>
       <c r="K20" t="n">
-        <v>10.34</v>
+        <v>6.39</v>
       </c>
       <c r="L20" t="n">
-        <v>23.76</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="21">
@@ -1322,42 +1322,42 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SUNTV</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Media Entertainment &amp; Publication</t>
+          <t>Automobile and Auto Components</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Smallcap</t>
+          <t>Largecap</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>605.6</v>
+        <v>37740</v>
       </c>
       <c r="F21" t="n">
-        <v>605.6</v>
+        <v>37740</v>
       </c>
       <c r="G21" t="n">
-        <v>17.23</v>
+        <v>102.13</v>
       </c>
       <c r="H21" t="n">
-        <v>2.18</v>
+        <v>1.61</v>
       </c>
       <c r="I21" t="n">
-        <v>3.98</v>
+        <v>0.8</v>
       </c>
       <c r="J21" t="n">
-        <v>12.78</v>
+        <v>6.09</v>
       </c>
       <c r="K21" t="n">
-        <v>9.550000000000001</v>
+        <v>2.89</v>
       </c>
       <c r="L21" t="n">
-        <v>7.47</v>
+        <v>-2.15</v>
       </c>
     </row>
     <row r="22">
@@ -1366,42 +1366,42 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SCHAEFFLER</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Automobile and Auto Components</t>
+          <t>Consumer Durables</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Midcap</t>
+          <t>Largecap</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>4124.8</v>
+        <v>2605.6</v>
       </c>
       <c r="F22" t="n">
-        <v>4124.8</v>
+        <v>2605.6</v>
       </c>
       <c r="G22" t="n">
-        <v>48.85</v>
+        <v>270.17</v>
       </c>
       <c r="H22" t="n">
-        <v>2.1</v>
+        <v>1.74</v>
       </c>
       <c r="I22" t="n">
-        <v>7.44</v>
+        <v>5.75</v>
       </c>
       <c r="J22" t="n">
-        <v>14.24</v>
+        <v>8.91</v>
       </c>
       <c r="K22" t="n">
-        <v>7.41</v>
+        <v>-5.78</v>
       </c>
       <c r="L22" t="n">
-        <v>3.12</v>
+        <v>5.42</v>
       </c>
     </row>
     <row r="23">
@@ -1410,42 +1410,42 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>SCHAEFFLER</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Chemicals</t>
+          <t>Automobile and Auto Components</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Largecap</t>
+          <t>Midcap</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>15439</v>
+        <v>4029.6</v>
       </c>
       <c r="F23" t="n">
-        <v>15439</v>
+        <v>4029.6</v>
       </c>
       <c r="G23" t="n">
-        <v>212.54</v>
+        <v>43.43</v>
       </c>
       <c r="H23" t="n">
-        <v>1.98</v>
+        <v>1.83</v>
       </c>
       <c r="I23" t="n">
-        <v>20.55</v>
+        <v>1.51</v>
       </c>
       <c r="J23" t="n">
-        <v>10.94</v>
+        <v>6.51</v>
       </c>
       <c r="K23" t="n">
-        <v>10.13</v>
+        <v>-2.47</v>
       </c>
       <c r="L23" t="n">
-        <v>4.66</v>
+        <v>4.07</v>
       </c>
     </row>
     <row r="24">
@@ -1454,42 +1454,42 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>LTFOODS</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Fast Moving Consumer Goods</t>
+          <t>Capital Goods</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Smallcap</t>
+          <t>Midcap</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>430.65</v>
+        <v>3856.3</v>
       </c>
       <c r="F24" t="n">
-        <v>430.65</v>
+        <v>3856.3</v>
       </c>
       <c r="G24" t="n">
-        <v>20.42</v>
+        <v>10.86</v>
       </c>
       <c r="H24" t="n">
-        <v>2.1</v>
+        <v>1.47</v>
       </c>
       <c r="I24" t="n">
-        <v>18.54</v>
+        <v>-1.76</v>
       </c>
       <c r="J24" t="n">
-        <v>21.21</v>
+        <v>-6.14</v>
       </c>
       <c r="K24" t="n">
-        <v>1.38</v>
+        <v>11.92</v>
       </c>
       <c r="L24" t="n">
-        <v>-11.09</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="25">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>HAL</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1508,32 +1508,32 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Midcap</t>
+          <t>Largecap</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>3949.6</v>
+        <v>4386.2</v>
       </c>
       <c r="F25" t="n">
-        <v>3949.6</v>
+        <v>4386.2</v>
       </c>
       <c r="G25" t="n">
-        <v>16.58</v>
+        <v>555.99</v>
       </c>
       <c r="H25" t="n">
-        <v>1.63</v>
+        <v>2.09</v>
       </c>
       <c r="I25" t="n">
-        <v>8.609999999999999</v>
+        <v>-0.04</v>
       </c>
       <c r="J25" t="n">
-        <v>2.8</v>
+        <v>7.01</v>
       </c>
       <c r="K25" t="n">
-        <v>17.54</v>
+        <v>-6.86</v>
       </c>
       <c r="L25" t="n">
-        <v>18.36</v>
+        <v>-0.07000000000000001</v>
       </c>
     </row>
     <row r="26">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AJANTPHARM</t>
+          <t>PFIZER</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1552,32 +1552,32 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Midcap</t>
+          <t>Smallcap</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>2822.7</v>
+        <v>4954.7</v>
       </c>
       <c r="F26" t="n">
-        <v>2822.7</v>
+        <v>4954.7</v>
       </c>
       <c r="G26" t="n">
-        <v>20.33</v>
+        <v>10.68</v>
       </c>
       <c r="H26" t="n">
-        <v>1.38</v>
+        <v>1.94</v>
       </c>
       <c r="I26" t="n">
-        <v>0.21</v>
+        <v>1.97</v>
       </c>
       <c r="J26" t="n">
-        <v>3.84</v>
+        <v>-0.12</v>
       </c>
       <c r="K26" t="n">
-        <v>19.27</v>
+        <v>-0.85</v>
       </c>
       <c r="L26" t="n">
-        <v>2.07</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="27">
@@ -1586,42 +1586,42 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Fast Moving Consumer Goods</t>
+          <t>Capital Goods</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Midcap</t>
+          <t>Largecap</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>775</v>
+        <v>423.65</v>
       </c>
       <c r="F27" t="n">
-        <v>775</v>
+        <v>423.65</v>
       </c>
       <c r="G27" t="n">
-        <v>133.83</v>
+        <v>500.19</v>
       </c>
       <c r="H27" t="n">
-        <v>1.09</v>
+        <v>1.38</v>
       </c>
       <c r="I27" t="n">
-        <v>4.1</v>
+        <v>-8.449999999999999</v>
       </c>
       <c r="J27" t="n">
-        <v>5.21</v>
+        <v>-2.76</v>
       </c>
       <c r="K27" t="n">
-        <v>7.63</v>
+        <v>0.17</v>
       </c>
       <c r="L27" t="n">
-        <v>12.79</v>
+        <v>10.88</v>
       </c>
     </row>
     <row r="28">
@@ -1630,12 +1630,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>3MINDIA</t>
+          <t>360ONE</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Diversified</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1644,28 +1644,28 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>33300</v>
+        <v>1093.8</v>
       </c>
       <c r="F28" t="n">
-        <v>33300</v>
+        <v>1093.8</v>
       </c>
       <c r="G28" t="n">
-        <v>19.83</v>
+        <v>130.32</v>
       </c>
       <c r="H28" t="n">
-        <v>2.31</v>
+        <v>1.92</v>
       </c>
       <c r="I28" t="n">
-        <v>10.56</v>
+        <v>-1.18</v>
       </c>
       <c r="J28" t="n">
-        <v>0.68</v>
+        <v>-3.36</v>
       </c>
       <c r="K28" t="n">
-        <v>11.99</v>
+        <v>2.82</v>
       </c>
       <c r="L28" t="n">
-        <v>7.44</v>
+        <v>3.79</v>
       </c>
     </row>
     <row r="29">
@@ -1674,42 +1674,42 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ASTRAL</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Capital Goods</t>
+          <t>Automobile and Auto Components</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Midcap</t>
+          <t>Largecap</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>1529.7</v>
+        <v>7014.5</v>
       </c>
       <c r="F29" t="n">
-        <v>1529.7</v>
+        <v>7014.5</v>
       </c>
       <c r="G29" t="n">
-        <v>145.6</v>
+        <v>321.25</v>
       </c>
       <c r="H29" t="n">
-        <v>1.7</v>
+        <v>1.23</v>
       </c>
       <c r="I29" t="n">
-        <v>-2.59</v>
+        <v>-2.43</v>
       </c>
       <c r="J29" t="n">
-        <v>5.29</v>
+        <v>-9.73</v>
       </c>
       <c r="K29" t="n">
-        <v>5.58</v>
+        <v>1.97</v>
       </c>
       <c r="L29" t="n">
-        <v>6.5</v>
+        <v>23.87</v>
       </c>
     </row>
     <row r="30">
@@ -1718,42 +1718,42 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>ASTRAL</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Capital Goods</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Largecap</t>
+          <t>Midcap</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>6502.5</v>
+        <v>1550.8</v>
       </c>
       <c r="F30" t="n">
-        <v>6502.5</v>
+        <v>1550.8</v>
       </c>
       <c r="G30" t="n">
-        <v>193.46</v>
+        <v>89.81</v>
       </c>
       <c r="H30" t="n">
-        <v>1.15</v>
+        <v>1.38</v>
       </c>
       <c r="I30" t="n">
-        <v>9.34</v>
+        <v>-3.38</v>
       </c>
       <c r="J30" t="n">
-        <v>7.37</v>
+        <v>-2.59</v>
       </c>
       <c r="K30" t="n">
-        <v>0.19</v>
+        <v>-2.17</v>
       </c>
       <c r="L30" t="n">
-        <v>-1.31</v>
+        <v>13.02</v>
       </c>
     </row>
     <row r="31">
@@ -1762,42 +1762,42 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>MUTHOOTFIN</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Capital Goods</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Largecap</t>
+          <t>Midcap</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>431.3</v>
+        <v>3311.4</v>
       </c>
       <c r="F31" t="n">
-        <v>431.3</v>
+        <v>3311.4</v>
       </c>
       <c r="G31" t="n">
-        <v>577.14</v>
+        <v>266.68</v>
       </c>
       <c r="H31" t="n">
-        <v>1.46</v>
+        <v>2.23</v>
       </c>
       <c r="I31" t="n">
-        <v>3.01</v>
+        <v>-7.28</v>
       </c>
       <c r="J31" t="n">
-        <v>-4.38</v>
+        <v>-15.1</v>
       </c>
       <c r="K31" t="n">
-        <v>4.74</v>
+        <v>0.44</v>
       </c>
       <c r="L31" t="n">
-        <v>9.85</v>
+        <v>27.57</v>
       </c>
     </row>
   </sheetData>
@@ -1811,7 +1811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1838,10 +1838,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
@@ -1851,10 +1851,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4">
@@ -1864,10 +1864,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C4" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
@@ -1894,36 +1894,36 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Automobile and Auto Components</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C8" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Metals &amp; Mining</t>
+          <t>Automobile and Auto Components</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -1933,10 +1933,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
@@ -1955,7 +1955,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Oil Gas &amp; Consumable Fuels</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1968,39 +1968,13 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Oil Gas &amp; Consumable Fuels</t>
+          <t>Metals &amp; Mining</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>1</v>
       </c>
       <c r="C13" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Media Entertainment &amp; Publication</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2015,7 +1989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H108"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2038,7 +2012,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2024,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2048,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
@@ -2098,7 +2072,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>biweekly: computed baseline as-of 2026-04-17 (n_ranked=36; archive cutoff 2026-04-17 00:00:00)</t>
+          <t>biweekly: baseline top 20 from ranked universe as-of 2026-05-01 (n_ranked=34); rebalance session 2026-05-15</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2084,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-05-12T19:34:17</t>
+          <t>2026-05-16T01:25:57</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2096,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2108,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-05-12T19:34:18</t>
+          <t>2026-05-16T01:25:59</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2155,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1) Current session — top 20 portfolio (this run, session 2026-05-01)</t>
+          <t>1) Current session — top 20 portfolio (this run, session 2026-05-15)</t>
         </is>
       </c>
     </row>
@@ -2205,75 +2179,79 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>7230</v>
+        <v>5392</v>
       </c>
       <c r="C19" t="n">
-        <v>3.27</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>5266.4</v>
+        <v>9152.5</v>
       </c>
       <c r="C20" t="n">
-        <v>2.44</v>
+        <v>12.85</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FINCABLES</t>
+          <t>ABSLAMC</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>990.55</v>
-      </c>
-      <c r="C21" t="inlineStr"/>
+        <v>1030.4</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ABSLAMC</t>
+          <t>KEI</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1015.2</v>
-      </c>
-      <c r="C22" t="inlineStr"/>
+        <v>5117.5</v>
+      </c>
+      <c r="C22" t="n">
+        <v>5.35</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>607.25</v>
+        <v>2140.4</v>
       </c>
       <c r="C23" t="n">
-        <v>2.26</v>
+        <v>4.75</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>KEI</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>4857.5</v>
+        <v>462.2</v>
       </c>
       <c r="C24" t="n">
-        <v>0.38</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="25">
@@ -2283,47 +2261,47 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>90.37</v>
+        <v>91.41</v>
       </c>
       <c r="C25" t="n">
-        <v>0.66</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>OFSS</t>
+          <t>GPIL</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>9455.610000000001</v>
+        <v>287.9</v>
       </c>
       <c r="C26" t="n">
-        <v>21.7</v>
+        <v>-2.83</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GPIL</t>
+          <t>AJANTPHARM</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>296.3</v>
+        <v>3177.2</v>
       </c>
       <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>TIMKEN</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>481.45</v>
+        <v>3531.2</v>
       </c>
       <c r="C28" t="n">
-        <v>9.73</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="29">
@@ -2333,131 +2311,125 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1458.6</v>
+        <v>1430.5</v>
       </c>
       <c r="C29" t="n">
-        <v>13.46</v>
+        <v>-1.93</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>ZYDUSLIFE</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2043.4</v>
-      </c>
-      <c r="C30" t="n">
-        <v>2.27</v>
-      </c>
+        <v>1011.7</v>
+      </c>
+      <c r="C30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>553.5</v>
-      </c>
-      <c r="C31" t="n">
-        <v>0.79</v>
-      </c>
+        <v>841.15</v>
+      </c>
+      <c r="C31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>8110.5</v>
+        <v>573.55</v>
       </c>
       <c r="C32" t="n">
-        <v>-0.88</v>
+        <v>-5.55</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TIMKEN</t>
+          <t>VBL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3428.8</v>
+        <v>503.8</v>
       </c>
       <c r="C33" t="n">
-        <v>-2.22</v>
+        <v>-1.93</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TIINDIA</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2947.9</v>
+        <v>10377.5</v>
       </c>
       <c r="C34" t="n">
-        <v>5.65</v>
+        <v>3.84</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>HINDZINC</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>595.95</v>
+        <v>6760.5</v>
       </c>
       <c r="C35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>VBL</t>
+          <t>TIINDIA</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>513.7</v>
+        <v>2850.3</v>
       </c>
       <c r="C36" t="n">
-        <v>8.5</v>
+        <v>-3.31</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>9994</v>
+        <v>523.25</v>
       </c>
       <c r="C37" t="n">
-        <v>2.26</v>
+        <v>-5.47</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SUNTV</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>605.6</v>
-      </c>
-      <c r="C38" t="n">
-        <v>-5.85</v>
-      </c>
+        <v>37740</v>
+      </c>
+      <c r="C38" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2) Previous baseline — IN/OUT symbols: Adj close at baseline session 2026-04-17 vs current session 2026-05-01</t>
+          <t>2) Entering top portfolio — new names vs previous baseline</t>
         </is>
       </c>
     </row>
@@ -2469,15 +2441,10 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Baseline_Adj_Close</t>
+          <t>Adj_Close</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
-        <is>
-          <t>Current_Adj_Close</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
         <is>
           <t>Pct_vs_baseline</t>
         </is>
@@ -2486,368 +2453,441 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>APARINDS</t>
+          <t>AJANTPHARM</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>11482</v>
-      </c>
-      <c r="C43" t="n">
-        <v>12331</v>
-      </c>
-      <c r="D43" t="n">
-        <v>7.39</v>
-      </c>
+        <v>3177.2</v>
+      </c>
+      <c r="C43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>593.85</v>
-      </c>
-      <c r="C44" t="n">
-        <v>607.25</v>
-      </c>
-      <c r="D44" t="n">
-        <v>2.26</v>
-      </c>
+        <v>37740</v>
+      </c>
+      <c r="C44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>7000.87</v>
-      </c>
-      <c r="C45" t="n">
-        <v>7230</v>
-      </c>
-      <c r="D45" t="n">
-        <v>3.27</v>
-      </c>
+        <v>6760.5</v>
+      </c>
+      <c r="C45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>5140.9</v>
-      </c>
-      <c r="C46" t="n">
-        <v>5266.4</v>
-      </c>
-      <c r="D46" t="n">
-        <v>2.44</v>
-      </c>
+        <v>841.15</v>
+      </c>
+      <c r="C46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>NMDC</t>
+          <t>ZYDUSLIFE</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>89.78</v>
-      </c>
-      <c r="C47" t="n">
-        <v>90.37</v>
-      </c>
-      <c r="D47" t="n">
-        <v>0.66</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>TIMKEN</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>3506.6</v>
-      </c>
-      <c r="C48" t="n">
-        <v>3428.8</v>
-      </c>
-      <c r="D48" t="n">
-        <v>-2.22</v>
-      </c>
+        <v>1011.7</v>
+      </c>
+      <c r="C47" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>549.15</v>
-      </c>
-      <c r="C49" t="n">
-        <v>553.5</v>
-      </c>
-      <c r="D49" t="n">
-        <v>0.79</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>KEI</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>4839.3</v>
-      </c>
-      <c r="C50" t="n">
-        <v>4857.5</v>
-      </c>
-      <c r="D50" t="n">
-        <v>0.38</v>
+          <t>3) Leaving top portfolio — names that dropped out of top vs previous baseline</t>
+        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SUNTV</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>643.25</v>
-      </c>
-      <c r="C51" t="n">
-        <v>605.6</v>
-      </c>
-      <c r="D51" t="n">
-        <v>-5.85</v>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Adj_Close</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Pct_vs_baseline</t>
+        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1998</v>
+        <v>6381</v>
       </c>
       <c r="C52" t="n">
-        <v>2043.4</v>
-      </c>
-      <c r="D52" t="n">
-        <v>2.27</v>
+        <v>-11.74</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>FINCABLES</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>462.75</v>
+        <v>1050.9</v>
       </c>
       <c r="C53" t="n">
-        <v>431.3</v>
-      </c>
-      <c r="D53" t="n">
-        <v>-6.8</v>
+        <v>6.09</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ASTRAL</t>
+          <t>HINDZINC</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1605</v>
+        <v>637.8</v>
       </c>
       <c r="C54" t="n">
-        <v>1529.7</v>
-      </c>
-      <c r="D54" t="n">
-        <v>-4.69</v>
+        <v>7.02</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>OFSS</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>438.75</v>
+        <v>9015</v>
       </c>
       <c r="C55" t="n">
-        <v>481.45</v>
-      </c>
-      <c r="D55" t="n">
-        <v>9.73</v>
+        <v>-4.66</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>SUNTV</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>15089</v>
+        <v>535.15</v>
       </c>
       <c r="C56" t="n">
-        <v>15439</v>
-      </c>
-      <c r="D56" t="n">
-        <v>2.32</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>POLYCAB</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>8182.5</v>
-      </c>
-      <c r="C57" t="n">
-        <v>8110.5</v>
-      </c>
-      <c r="D57" t="n">
-        <v>-0.88</v>
+        <v>-11.63</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>LTFOODS</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>422</v>
-      </c>
-      <c r="C58" t="n">
-        <v>430.65</v>
-      </c>
-      <c r="D58" t="n">
-        <v>2.05</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>AIAENG</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>3961.5</v>
-      </c>
-      <c r="C59" t="n">
-        <v>3949.6</v>
-      </c>
-      <c r="D59" t="n">
-        <v>-0.3</v>
+          <t>4) Prior baseline top 20 — baseline session 2026-05-01 vs 2026-05-15: adj. close, % change, rank, exit monitor</t>
+        </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>AJANTPHARM</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>2790.2</v>
-      </c>
-      <c r="C60" t="n">
-        <v>2822.7</v>
-      </c>
-      <c r="D60" t="n">
-        <v>1.16</v>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Baseline_Adj_Close</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Current_Adj_Close</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Pct_vs_baseline</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Current_Rank</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>In_top_portfolio</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Within_exit_rank_band</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>TIINDIA</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>2790.2</v>
+        <v>7230</v>
       </c>
       <c r="C61" t="n">
-        <v>2947.9</v>
+        <v>6381</v>
       </c>
       <c r="D61" t="n">
-        <v>5.65</v>
+        <v>-11.74</v>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Failed screen — not in ranked universe this run</t>
+        </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>9773.5</v>
+        <v>5266.4</v>
       </c>
       <c r="C62" t="n">
-        <v>9994</v>
+        <v>5392</v>
       </c>
       <c r="D62" t="n">
-        <v>2.26</v>
+        <v>2.38</v>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>FINCABLES</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>990.55</v>
+      </c>
+      <c r="C63" t="n">
+        <v>1050.9</v>
+      </c>
+      <c r="D63" t="n">
+        <v>6.09</v>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Failed screen — not in ranked universe this run</t>
+        </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>3) Entering top portfolio — new names vs previous baseline</t>
-        </is>
-      </c>
+          <t>ABSLAMC</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>1015.2</v>
+      </c>
+      <c r="C64" t="n">
+        <v>1030.4</v>
+      </c>
+      <c r="D64" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E64" t="n">
+        <v>3</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>SONACOMS</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>607.25</v>
+      </c>
+      <c r="C65" t="n">
+        <v>573.55</v>
+      </c>
+      <c r="D65" t="n">
+        <v>-5.55</v>
+      </c>
+      <c r="E65" t="n">
+        <v>14</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Symbol</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Adj_Close</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Pct_vs_baseline</t>
-        </is>
-      </c>
+          <t>KEI</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>4857.5</v>
+      </c>
+      <c r="C66" t="n">
+        <v>5117.5</v>
+      </c>
+      <c r="D66" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="E66" t="n">
+        <v>4</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ABSLAMC</t>
+          <t>NMDC</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1015.2</v>
-      </c>
-      <c r="C67" t="inlineStr"/>
+        <v>90.37</v>
+      </c>
+      <c r="C67" t="n">
+        <v>91.41</v>
+      </c>
+      <c r="D67" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E67" t="n">
+        <v>7</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>FINCABLES</t>
+          <t>OFSS</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>990.55</v>
-      </c>
-      <c r="C68" t="inlineStr"/>
+        <v>9455.610000000001</v>
+      </c>
+      <c r="C68" t="n">
+        <v>9015</v>
+      </c>
+      <c r="D68" t="n">
+        <v>-4.66</v>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Failed screen — not in ranked universe this run</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2858,18 +2898,56 @@
       <c r="B69" t="n">
         <v>296.3</v>
       </c>
-      <c r="C69" t="inlineStr"/>
+      <c r="C69" t="n">
+        <v>287.9</v>
+      </c>
+      <c r="D69" t="n">
+        <v>-2.83</v>
+      </c>
+      <c r="E69" t="n">
+        <v>8</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>HINDZINC</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>595.95</v>
-      </c>
-      <c r="C70" t="inlineStr"/>
+        <v>481.45</v>
+      </c>
+      <c r="C70" t="n">
+        <v>462.2</v>
+      </c>
+      <c r="D70" t="n">
+        <v>-4</v>
+      </c>
+      <c r="E70" t="n">
+        <v>6</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2881,824 +2959,299 @@
         <v>1458.6</v>
       </c>
       <c r="C71" t="n">
-        <v>13.46</v>
-      </c>
+        <v>1430.5</v>
+      </c>
+      <c r="D71" t="n">
+        <v>-1.93</v>
+      </c>
+      <c r="E71" t="n">
+        <v>11</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>OFSS</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>9455.610000000001</v>
+        <v>2043.4</v>
       </c>
       <c r="C72" t="n">
-        <v>21.7</v>
-      </c>
+        <v>2140.4</v>
+      </c>
+      <c r="D72" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="E72" t="n">
+        <v>5</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>VBL</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>513.7</v>
+        <v>553.5</v>
       </c>
       <c r="C73" t="n">
-        <v>8.5</v>
-      </c>
+        <v>523.25</v>
+      </c>
+      <c r="D73" t="n">
+        <v>-5.47</v>
+      </c>
+      <c r="E73" t="n">
+        <v>19</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>8110.5</v>
+      </c>
+      <c r="C74" t="n">
+        <v>9152.5</v>
+      </c>
+      <c r="D74" t="n">
+        <v>12.85</v>
+      </c>
+      <c r="E74" t="n">
+        <v>2</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>4) Leaving top portfolio — names that dropped out of top vs previous baseline</t>
-        </is>
-      </c>
+          <t>TIMKEN</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>3428.8</v>
+      </c>
+      <c r="C75" t="n">
+        <v>3531.2</v>
+      </c>
+      <c r="D75" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E75" t="n">
+        <v>10</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>TIINDIA</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>2947.9</v>
+      </c>
+      <c r="C76" t="n">
+        <v>2850.3</v>
+      </c>
+      <c r="D76" t="n">
+        <v>-3.31</v>
+      </c>
+      <c r="E76" t="n">
+        <v>18</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Symbol</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Adj_Close</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Pct_vs_baseline</t>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>595.95</v>
+      </c>
+      <c r="C77" t="n">
+        <v>637.8</v>
+      </c>
+      <c r="D77" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Failed screen — not in ranked universe this run</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>VBL</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>3949.6</v>
+        <v>513.7</v>
       </c>
       <c r="C78" t="n">
-        <v>-0.3</v>
-      </c>
+        <v>503.8</v>
+      </c>
+      <c r="D78" t="n">
+        <v>-1.93</v>
+      </c>
+      <c r="E78" t="n">
+        <v>15</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>AJANTPHARM</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>2822.7</v>
+        <v>9994</v>
       </c>
       <c r="C79" t="n">
-        <v>1.16</v>
-      </c>
+        <v>10377.5</v>
+      </c>
+      <c r="D79" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="E79" t="n">
+        <v>16</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>APARINDS</t>
+          <t>SUNTV</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>12331</v>
+        <v>605.6</v>
       </c>
       <c r="C80" t="n">
-        <v>7.39</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>ASTRAL</t>
-        </is>
-      </c>
-      <c r="B81" t="n">
-        <v>1529.7</v>
-      </c>
-      <c r="C81" t="n">
-        <v>-4.69</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>BEL</t>
-        </is>
-      </c>
-      <c r="B82" t="n">
-        <v>431.3</v>
-      </c>
-      <c r="C82" t="n">
-        <v>-6.8</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>LTFOODS</t>
-        </is>
-      </c>
-      <c r="B83" t="n">
-        <v>430.65</v>
-      </c>
-      <c r="C83" t="n">
-        <v>2.05</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>SOLARINDS</t>
-        </is>
-      </c>
-      <c r="B84" t="n">
-        <v>15439</v>
-      </c>
-      <c r="C84" t="n">
-        <v>2.32</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>5) Each previous baseline name — baseline vs current adj. close, rank at 2026-05-01 (exit monitor)</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Symbol</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>Baseline_Adj_Close</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Current_Adj_Close</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>Pct_vs_baseline</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Current_Rank</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>In_top_portfolio</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>Within_exit_rank_band</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>APARINDS</t>
-        </is>
-      </c>
-      <c r="B89" t="n">
-        <v>11482</v>
-      </c>
-      <c r="C89" t="n">
-        <v>12331</v>
-      </c>
-      <c r="D89" t="n">
-        <v>7.39</v>
-      </c>
-      <c r="E89" t="inlineStr"/>
-      <c r="F89" t="inlineStr">
+        <v>535.15</v>
+      </c>
+      <c r="D80" t="n">
+        <v>-11.63</v>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr">
+      <c r="G80" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr">
+      <c r="H80" t="inlineStr">
         <is>
           <t>Failed screen — not in ranked universe this run</t>
         </is>
       </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>SONACOMS</t>
-        </is>
-      </c>
-      <c r="B90" t="n">
-        <v>593.85</v>
-      </c>
-      <c r="C90" t="n">
-        <v>607.25</v>
-      </c>
-      <c r="D90" t="n">
-        <v>2.26</v>
-      </c>
-      <c r="E90" t="n">
-        <v>5</v>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>ABB</t>
-        </is>
-      </c>
-      <c r="B91" t="n">
-        <v>7000.87</v>
-      </c>
-      <c r="C91" t="n">
-        <v>7230</v>
-      </c>
-      <c r="D91" t="n">
-        <v>3.27</v>
-      </c>
-      <c r="E91" t="n">
-        <v>1</v>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>CUMMINSIND</t>
-        </is>
-      </c>
-      <c r="B92" t="n">
-        <v>5140.9</v>
-      </c>
-      <c r="C92" t="n">
-        <v>5266.4</v>
-      </c>
-      <c r="D92" t="n">
-        <v>2.44</v>
-      </c>
-      <c r="E92" t="n">
-        <v>2</v>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H92" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>NMDC</t>
-        </is>
-      </c>
-      <c r="B93" t="n">
-        <v>89.78</v>
-      </c>
-      <c r="C93" t="n">
-        <v>90.37</v>
-      </c>
-      <c r="D93" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="E93" t="n">
-        <v>7</v>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H93" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>TIMKEN</t>
-        </is>
-      </c>
-      <c r="B94" t="n">
-        <v>3506.6</v>
-      </c>
-      <c r="C94" t="n">
-        <v>3428.8</v>
-      </c>
-      <c r="D94" t="n">
-        <v>-2.22</v>
-      </c>
-      <c r="E94" t="n">
-        <v>15</v>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H94" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>ELGIEQUIP</t>
-        </is>
-      </c>
-      <c r="B95" t="n">
-        <v>549.15</v>
-      </c>
-      <c r="C95" t="n">
-        <v>553.5</v>
-      </c>
-      <c r="D95" t="n">
-        <v>0.79</v>
-      </c>
-      <c r="E95" t="n">
-        <v>13</v>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>KEI</t>
-        </is>
-      </c>
-      <c r="B96" t="n">
-        <v>4839.3</v>
-      </c>
-      <c r="C96" t="n">
-        <v>4857.5</v>
-      </c>
-      <c r="D96" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="E96" t="n">
-        <v>6</v>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H96" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>SUNTV</t>
-        </is>
-      </c>
-      <c r="B97" t="n">
-        <v>643.25</v>
-      </c>
-      <c r="C97" t="n">
-        <v>605.6</v>
-      </c>
-      <c r="D97" t="n">
-        <v>-5.85</v>
-      </c>
-      <c r="E97" t="n">
-        <v>20</v>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H97" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>JBCHEPHARM</t>
-        </is>
-      </c>
-      <c r="B98" t="n">
-        <v>1998</v>
-      </c>
-      <c r="C98" t="n">
-        <v>2043.4</v>
-      </c>
-      <c r="D98" t="n">
-        <v>2.27</v>
-      </c>
-      <c r="E98" t="n">
-        <v>12</v>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H98" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>BEL</t>
-        </is>
-      </c>
-      <c r="B99" t="n">
-        <v>462.75</v>
-      </c>
-      <c r="C99" t="n">
-        <v>431.3</v>
-      </c>
-      <c r="D99" t="n">
-        <v>-6.8</v>
-      </c>
-      <c r="E99" t="n">
-        <v>30</v>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>Below top 20 (universe rank 30)</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>ASTRAL</t>
-        </is>
-      </c>
-      <c r="B100" t="n">
-        <v>1605</v>
-      </c>
-      <c r="C100" t="n">
-        <v>1529.7</v>
-      </c>
-      <c r="D100" t="n">
-        <v>-4.69</v>
-      </c>
-      <c r="E100" t="n">
-        <v>28</v>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>Below top 20 (universe rank 28)</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>COALINDIA</t>
-        </is>
-      </c>
-      <c r="B101" t="n">
-        <v>438.75</v>
-      </c>
-      <c r="C101" t="n">
-        <v>481.45</v>
-      </c>
-      <c r="D101" t="n">
-        <v>9.73</v>
-      </c>
-      <c r="E101" t="n">
-        <v>10</v>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H101" t="inlineStr"/>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>SOLARINDS</t>
-        </is>
-      </c>
-      <c r="B102" t="n">
-        <v>15089</v>
-      </c>
-      <c r="C102" t="n">
-        <v>15439</v>
-      </c>
-      <c r="D102" t="n">
-        <v>2.32</v>
-      </c>
-      <c r="E102" t="n">
-        <v>22</v>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G102" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>Below top 20 (universe rank 22)</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>POLYCAB</t>
-        </is>
-      </c>
-      <c r="B103" t="n">
-        <v>8182.5</v>
-      </c>
-      <c r="C103" t="n">
-        <v>8110.5</v>
-      </c>
-      <c r="D103" t="n">
-        <v>-0.88</v>
-      </c>
-      <c r="E103" t="n">
-        <v>14</v>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H103" t="inlineStr"/>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>LTFOODS</t>
-        </is>
-      </c>
-      <c r="B104" t="n">
-        <v>422</v>
-      </c>
-      <c r="C104" t="n">
-        <v>430.65</v>
-      </c>
-      <c r="D104" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="E104" t="n">
-        <v>23</v>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H104" t="inlineStr">
-        <is>
-          <t>Below top 20 (universe rank 23)</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>AIAENG</t>
-        </is>
-      </c>
-      <c r="B105" t="n">
-        <v>3961.5</v>
-      </c>
-      <c r="C105" t="n">
-        <v>3949.6</v>
-      </c>
-      <c r="D105" t="n">
-        <v>-0.3</v>
-      </c>
-      <c r="E105" t="n">
-        <v>24</v>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>Below top 20 (universe rank 24)</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>AJANTPHARM</t>
-        </is>
-      </c>
-      <c r="B106" t="n">
-        <v>2790.2</v>
-      </c>
-      <c r="C106" t="n">
-        <v>2822.7</v>
-      </c>
-      <c r="D106" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="E106" t="n">
-        <v>25</v>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H106" t="inlineStr">
-        <is>
-          <t>Below top 20 (universe rank 25)</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>TIINDIA</t>
-        </is>
-      </c>
-      <c r="B107" t="n">
-        <v>2790.2</v>
-      </c>
-      <c r="C107" t="n">
-        <v>2947.9</v>
-      </c>
-      <c r="D107" t="n">
-        <v>5.65</v>
-      </c>
-      <c r="E107" t="n">
-        <v>16</v>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H107" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>BAJAJ-AUTO</t>
-        </is>
-      </c>
-      <c r="B108" t="n">
-        <v>9773.5</v>
-      </c>
-      <c r="C108" t="n">
-        <v>9994</v>
-      </c>
-      <c r="D108" t="n">
-        <v>2.26</v>
-      </c>
-      <c r="E108" t="n">
-        <v>19</v>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H108" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>